<commit_message>
Port shared MDF convention to script 09 and figures; correct UGGA datasheet precision
- campaign MAD sigma per constant-interval run; closure length in seconds
  (YMF record is 5 s, LGR2 10 s); reference method = 95 % two-sided
- figures 1/2 and sensitivity use the reference flag from the compiled results
  instead of hard-coded 1.645 x 1.241 ppb / nb.obs
- x3*t variant relabelled (not Christiansen 2015); datasheet spec-equivalent at
  logging interval added to precision_comparison.csv
- 00_setup.R: GLA131 datasheet values (0.35 ppm, 0.9 ppb); goFlux steps not re-run
- comment_response_stats.R added; private drafts/worklogs gitignored

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data processing/goFlux_reprocessing/ymf_black_oak/results/ymf_black_oak_flux_compiled_with_mdf.xlsx
+++ b/data processing/goFlux_reprocessing/ymf_black_oak/results/ymf_black_oak_flux_compiled_with_mdf.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="153">
   <si>
     <t xml:space="preserve">instrument</t>
   </si>
@@ -158,13 +158,22 @@
     <t xml:space="preserve">n_meas_pts</t>
   </si>
   <si>
+    <t xml:space="preserve">dt_s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">t_sec</t>
+  </si>
+  <si>
     <t xml:space="preserve">flat_sd_CO2</t>
   </si>
   <si>
     <t xml:space="preserve">flat_sd_CH4</t>
   </si>
   <si>
-    <t xml:space="preserve">t_sec</t>
+    <t xml:space="preserve">mad_sd_CO2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mad_sd_CH4</t>
   </si>
   <si>
     <t xml:space="preserve">CO2_MDF_goflux</t>
@@ -1052,19 +1061,28 @@
       <c r="CI1" t="s">
         <v>86</v>
       </c>
+      <c r="CJ1" t="s">
+        <v>87</v>
+      </c>
+      <c r="CK1" t="s">
+        <v>88</v>
+      </c>
+      <c r="CL1" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E2" t="n">
         <v>12.9</v>
@@ -1075,16 +1093,16 @@
       </c>
       <c r="H2"/>
       <c r="I2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="J2" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="L2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="M2" t="n">
         <v>300</v>
@@ -1093,10 +1111,10 @@
         <v>1.14173417378919</v>
       </c>
       <c r="O2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="P2" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="Q2" t="n">
         <v>1.09028443267916</v>
@@ -1120,10 +1138,10 @@
         <v>1.12969676375376</v>
       </c>
       <c r="X2" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="Y2" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="Z2" t="n">
         <v>48</v>
@@ -1141,10 +1159,10 @@
         <v>-0.00484885854885949</v>
       </c>
       <c r="AE2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="AF2" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="AG2" t="n">
         <v>-0.00403629265498706</v>
@@ -1168,10 +1186,10 @@
         <v>1.6590185751789</v>
       </c>
       <c r="AN2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="AO2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="AP2" t="n">
         <v>48</v>
@@ -1195,64 +1213,64 @@
         <v>48</v>
       </c>
       <c r="AW2" t="n">
+        <v>5</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>239</v>
+      </c>
+      <c r="AY2" t="n">
         <v>1.10388215394272</v>
       </c>
-      <c r="AX2" t="n">
+      <c r="AZ2" t="n">
         <v>1.24063893013517</v>
       </c>
-      <c r="AY2" t="n">
-        <v>48</v>
-      </c>
-      <c r="AZ2" t="n">
-        <v>0.0169876847148722</v>
-      </c>
       <c r="BA2" t="n">
-        <v>0.0436826178382427</v>
+        <v>1.04228663609991</v>
       </c>
       <c r="BB2" t="n">
-        <v>0.138008533048349</v>
+        <v>1.40029850566019</v>
       </c>
       <c r="BC2" t="n">
-        <v>0.155106012158172</v>
+        <v>0.00341175257871909</v>
       </c>
       <c r="BD2" t="n">
-        <v>0.105011521517088</v>
+        <v>0.00877307805956339</v>
       </c>
       <c r="BE2" t="n">
-        <v>0.118021096039557</v>
+        <v>0.0261706032242944</v>
       </c>
       <c r="BF2" t="n">
-        <v>0.0881284469518497</v>
+        <v>0.0351598642042769</v>
       </c>
       <c r="BG2" t="n">
-        <v>0.0990464260612465</v>
+        <v>0.0199133691439236</v>
       </c>
       <c r="BH2" t="n">
-        <v>0.266547745086996</v>
+        <v>0.0267533518027599</v>
       </c>
       <c r="BI2" t="n">
-        <v>0.652361021305115</v>
+        <v>0.0167118261965884</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.199676251919299</v>
+        <v>0.0224521205965961</v>
       </c>
       <c r="BK2" t="n">
-        <v>0.488696700810343</v>
+        <v>0.053532601523748</v>
       </c>
       <c r="BL2" t="n">
-        <v>0.166520618259721</v>
+        <v>0.131018113065462</v>
       </c>
       <c r="BM2" t="n">
-        <v>0.407550101618064</v>
-      </c>
-      <c r="BN2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP2" t="b">
-        <v>0</v>
+        <v>0.0401023434817001</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>0.0981482913761359</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>0.0334434714496511</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>0.0818510664337534</v>
       </c>
       <c r="BQ2" t="b">
         <v>0</v>
@@ -1273,13 +1291,13 @@
         <v>0</v>
       </c>
       <c r="BW2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BX2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BY2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BZ2" t="b">
         <v>1</v>
@@ -1299,31 +1317,40 @@
       <c r="CE2" t="b">
         <v>1</v>
       </c>
-      <c r="CF2" t="n">
+      <c r="CF2" t="b">
+        <v>1</v>
+      </c>
+      <c r="CG2" t="b">
+        <v>1</v>
+      </c>
+      <c r="CH2" t="b">
+        <v>1</v>
+      </c>
+      <c r="CI2" t="n">
         <v>-0.0160211732658191</v>
       </c>
-      <c r="CG2" t="n">
+      <c r="CJ2" t="n">
         <v>0.998747896186046</v>
       </c>
-      <c r="CH2" t="n">
-        <v>0.080927644909931</v>
-      </c>
-      <c r="CI2" t="n">
-        <v>0.0599159725240499</v>
+      <c r="CK2" t="n">
+        <v>0.0162532508605719</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>0.298331613192665</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E3" t="n">
         <v>12.9</v>
@@ -1336,16 +1363,16 @@
       </c>
       <c r="H3"/>
       <c r="I3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="J3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="K3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="L3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="M3" t="n">
         <v>300</v>
@@ -1354,10 +1381,10 @@
         <v>1.3307836151745</v>
       </c>
       <c r="O3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="P3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="Q3" t="n">
         <v>1.27234696475888</v>
@@ -1381,10 +1408,10 @@
         <v>0.899074238592826</v>
       </c>
       <c r="X3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="Y3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="Z3" t="n">
         <v>77</v>
@@ -1402,10 +1429,10 @@
         <v>0.046013949999614</v>
       </c>
       <c r="AE3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="AF3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="AG3" t="n">
         <v>0.0387741109187982</v>
@@ -1429,10 +1456,10 @@
         <v>1.20687400068568</v>
       </c>
       <c r="AN3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AO3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AP3" t="n">
         <v>77</v>
@@ -1456,64 +1483,64 @@
         <v>77</v>
       </c>
       <c r="AW3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>383</v>
+      </c>
+      <c r="AY3" t="n">
         <v>1.10388215394272</v>
       </c>
-      <c r="AX3" t="n">
+      <c r="AZ3" t="n">
         <v>1.24063893013517</v>
       </c>
-      <c r="AY3" t="n">
-        <v>77</v>
-      </c>
-      <c r="AZ3" t="n">
-        <v>0.0105909502488075</v>
-      </c>
       <c r="BA3" t="n">
-        <v>0.027233872068362</v>
+        <v>1.04228663609991</v>
       </c>
       <c r="BB3" t="n">
-        <v>0.0860412429332613</v>
+        <v>1.40029850566019</v>
       </c>
       <c r="BC3" t="n">
-        <v>0.0967006443567896</v>
+        <v>0.00212925109440776</v>
       </c>
       <c r="BD3" t="n">
-        <v>0.065469298412713</v>
+        <v>0.00547521709990568</v>
       </c>
       <c r="BE3" t="n">
-        <v>0.0735801009639868</v>
+        <v>0.0163328917531181</v>
       </c>
       <c r="BF3" t="n">
-        <v>0.0549435672275326</v>
+        <v>0.0219430271125616</v>
       </c>
       <c r="BG3" t="n">
-        <v>0.0617503673009946</v>
+        <v>0.0124277954115196</v>
       </c>
       <c r="BH3" t="n">
-        <v>0.148821568610144</v>
+        <v>0.0166965810945439</v>
       </c>
       <c r="BI3" t="n">
-        <v>0.273820471546098</v>
+        <v>0.0104297346884391</v>
       </c>
       <c r="BJ3" t="n">
-        <v>0.112171648428468</v>
+        <v>0.0140122125649644</v>
       </c>
       <c r="BK3" t="n">
-        <v>0.206387380227442</v>
+        <v>0.0299197409477313</v>
       </c>
       <c r="BL3" t="n">
-        <v>0.0937770731711071</v>
+        <v>0.0550500686920354</v>
       </c>
       <c r="BM3" t="n">
-        <v>0.172542747907679</v>
-      </c>
-      <c r="BN3" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO3" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP3" t="b">
-        <v>0</v>
+        <v>0.0225514802323552</v>
+      </c>
+      <c r="BN3" t="n">
+        <v>0.0414930242232717</v>
+      </c>
+      <c r="BO3" t="n">
+        <v>0.0188533541362278</v>
+      </c>
+      <c r="BP3" t="n">
+        <v>0.0346887508848337</v>
       </c>
       <c r="BQ3" t="b">
         <v>0</v>
@@ -1537,22 +1564,22 @@
         <v>0</v>
       </c>
       <c r="BX3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BY3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BZ3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CA3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CB3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CC3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CD3" t="b">
         <v>1</v>
@@ -1560,31 +1587,40 @@
       <c r="CE3" t="b">
         <v>0</v>
       </c>
-      <c r="CF3" t="n">
+      <c r="CF3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG3" t="b">
+        <v>1</v>
+      </c>
+      <c r="CH3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI3" t="n">
         <v>0.695258815852541</v>
       </c>
-      <c r="CG3" t="n">
+      <c r="CJ3" t="n">
         <v>0.99977497116895</v>
       </c>
-      <c r="CH3" t="n">
-        <v>0.0345342698771411</v>
-      </c>
-      <c r="CI3" t="n">
-        <v>1.33241415449966</v>
+      <c r="CK3" t="n">
+        <v>0.00694292109801531</v>
+      </c>
+      <c r="CL3" t="n">
+        <v>6.62746261264117</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E4" t="n">
         <v>10.6</v>
@@ -1597,16 +1633,16 @@
       </c>
       <c r="H4"/>
       <c r="I4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="J4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L4" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="M4" t="n">
         <v>600</v>
@@ -1615,10 +1651,10 @@
         <v>1.1261297916822</v>
       </c>
       <c r="O4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="P4" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="Q4" t="n">
         <v>1.01572817524315</v>
@@ -1642,10 +1678,10 @@
         <v>1.40769764878489</v>
       </c>
       <c r="X4" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="Y4" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="Z4" t="n">
         <v>149</v>
@@ -1663,10 +1699,10 @@
         <v>0.0314898091802709</v>
       </c>
       <c r="AE4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="AF4" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="AG4" t="n">
         <v>0.0272394087536914</v>
@@ -1690,10 +1726,10 @@
         <v>1.75863641061905</v>
       </c>
       <c r="AN4" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AO4" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AP4" t="n">
         <v>149</v>
@@ -1717,64 +1753,64 @@
         <v>149</v>
       </c>
       <c r="AW4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>741</v>
+      </c>
+      <c r="AY4" t="n">
         <v>1.10388215394272</v>
       </c>
-      <c r="AX4" t="n">
+      <c r="AZ4" t="n">
         <v>1.24063893013517</v>
       </c>
-      <c r="AY4" t="n">
-        <v>149</v>
-      </c>
-      <c r="AZ4" t="n">
-        <v>0.00548708239664158</v>
-      </c>
       <c r="BA4" t="n">
-        <v>0.0141096404485069</v>
+        <v>1.04228663609991</v>
       </c>
       <c r="BB4" t="n">
-        <v>0.0445772455155683</v>
+        <v>1.40029850566019</v>
       </c>
       <c r="BC4" t="n">
-        <v>0.0500997918910802</v>
+        <v>0.00110334045492523</v>
       </c>
       <c r="BD4" t="n">
-        <v>0.0339190937924878</v>
+        <v>0.00283716116980773</v>
       </c>
       <c r="BE4" t="n">
-        <v>0.0381212324916797</v>
+        <v>0.00846341714439373</v>
       </c>
       <c r="BF4" t="n">
-        <v>0.0284658008450974</v>
+        <v>0.0113704905825324</v>
       </c>
       <c r="BG4" t="n">
-        <v>0.0319923468096351</v>
+        <v>0.00643986492672325</v>
       </c>
       <c r="BH4" t="n">
-        <v>0.11138257299646</v>
+        <v>0.00865187456234416</v>
       </c>
       <c r="BI4" t="n">
-        <v>0.165465728935058</v>
+        <v>0.00540450501404703</v>
       </c>
       <c r="BJ4" t="n">
-        <v>0.0843464656044522</v>
+        <v>0.00726088201928903</v>
       </c>
       <c r="BK4" t="n">
-        <v>0.125301912488411</v>
+        <v>0.0223967656902464</v>
       </c>
       <c r="BL4" t="n">
-        <v>0.0706482759480357</v>
+        <v>0.0332717862500995</v>
       </c>
       <c r="BM4" t="n">
-        <v>0.104952401109628</v>
-      </c>
-      <c r="BN4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP4" t="b">
-        <v>0</v>
+        <v>0.0169603554319344</v>
+      </c>
+      <c r="BN4" t="n">
+        <v>0.0251956612156184</v>
+      </c>
+      <c r="BO4" t="n">
+        <v>0.0142059286319262</v>
+      </c>
+      <c r="BP4" t="n">
+        <v>0.0211037891569967</v>
       </c>
       <c r="BQ4" t="b">
         <v>0</v>
@@ -1798,22 +1834,22 @@
         <v>0</v>
       </c>
       <c r="BX4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BY4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BZ4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CA4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CB4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CC4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CD4" t="b">
         <v>1</v>
@@ -1821,31 +1857,40 @@
       <c r="CE4" t="b">
         <v>0</v>
       </c>
-      <c r="CF4" t="n">
+      <c r="CF4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG4" t="b">
+        <v>1</v>
+      </c>
+      <c r="CH4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI4" t="n">
         <v>0.665931303103025</v>
       </c>
-      <c r="CG4" t="n">
+      <c r="CJ4" t="n">
         <v>0.999769549580697</v>
       </c>
-      <c r="CH4" t="n">
-        <v>0.0211348042636478</v>
-      </c>
-      <c r="CI4" t="n">
-        <v>1.48995035806571</v>
+      <c r="CK4" t="n">
+        <v>0.00424977845517345</v>
+      </c>
+      <c r="CL4" t="n">
+        <v>7.40975312299795</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B5" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C5" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D5" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E5" t="n">
         <v>12.9</v>
@@ -1858,16 +1903,16 @@
       </c>
       <c r="H5"/>
       <c r="I5" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="J5" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="K5" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="L5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="M5" t="n">
         <v>300</v>
@@ -1876,10 +1921,10 @@
         <v>1.20842158337</v>
       </c>
       <c r="O5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="P5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="Q5" t="n">
         <v>1.12550151487279</v>
@@ -1903,10 +1948,10 @@
         <v>2.27421231286376</v>
       </c>
       <c r="X5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="Y5" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="Z5" t="n">
         <v>69</v>
@@ -1924,10 +1969,10 @@
         <v>0.0384520122066485</v>
       </c>
       <c r="AE5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="AF5" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="AG5" t="n">
         <v>0.0384203355769582</v>
@@ -1951,10 +1996,10 @@
         <v>1.61678069534197</v>
       </c>
       <c r="AN5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AO5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AP5" t="n">
         <v>69</v>
@@ -1978,64 +2023,64 @@
         <v>69</v>
       </c>
       <c r="AW5" t="n">
+        <v>5</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>343</v>
+      </c>
+      <c r="AY5" t="n">
         <v>1.10388215394272</v>
       </c>
-      <c r="AX5" t="n">
+      <c r="AZ5" t="n">
         <v>1.24063893013517</v>
       </c>
-      <c r="AY5" t="n">
-        <v>69</v>
-      </c>
-      <c r="AZ5" t="n">
-        <v>0.0118306464064284</v>
-      </c>
       <c r="BA5" t="n">
-        <v>0.0304216621879589</v>
+        <v>1.04228663609991</v>
       </c>
       <c r="BB5" t="n">
-        <v>0.0961125770208999</v>
+        <v>1.40029850566019</v>
       </c>
       <c r="BC5" t="n">
-        <v>0.108019686976415</v>
+        <v>0.00237992595347978</v>
       </c>
       <c r="BD5" t="n">
-        <v>0.073132636996852</v>
+        <v>0.00611980959466228</v>
       </c>
       <c r="BE5" t="n">
-        <v>0.0821928284624179</v>
+        <v>0.0182557487375312</v>
       </c>
       <c r="BF5" t="n">
-        <v>0.0613748437020522</v>
+        <v>0.0245263603997917</v>
       </c>
       <c r="BG5" t="n">
-        <v>0.0689783960686066</v>
+        <v>0.0138909088374281</v>
       </c>
       <c r="BH5" t="n">
-        <v>0.291497849523514</v>
+        <v>0.0186622549053272</v>
       </c>
       <c r="BI5" t="n">
-        <v>0.342222766508585</v>
+        <v>0.011657618182335</v>
       </c>
       <c r="BJ5" t="n">
-        <v>0.21945829162363</v>
+        <v>0.0156618580291535</v>
       </c>
       <c r="BK5" t="n">
-        <v>0.257647265032835</v>
+        <v>0.0586395090878207</v>
       </c>
       <c r="BL5" t="n">
-        <v>0.183385014514273</v>
+        <v>0.0688436469069749</v>
       </c>
       <c r="BM5" t="n">
-        <v>0.215296706668256</v>
-      </c>
-      <c r="BN5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP5" t="b">
-        <v>0</v>
+        <v>0.0441475863616049</v>
+      </c>
+      <c r="BN5" t="n">
+        <v>0.0518299162894042</v>
+      </c>
+      <c r="BO5" t="n">
+        <v>0.0368908629780899</v>
+      </c>
+      <c r="BP5" t="n">
+        <v>0.0433104162102322</v>
       </c>
       <c r="BQ5" t="b">
         <v>0</v>
@@ -2059,54 +2104,63 @@
         <v>0</v>
       </c>
       <c r="BX5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BY5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BZ5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CA5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CB5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CC5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CD5" t="b">
         <v>1</v>
       </c>
       <c r="CE5" t="b">
-        <v>0</v>
-      </c>
-      <c r="CF5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF5" t="b">
+        <v>1</v>
+      </c>
+      <c r="CG5" t="b">
+        <v>1</v>
+      </c>
+      <c r="CH5" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI5" t="n">
         <v>0.496975719496566</v>
       </c>
-      <c r="CG5" t="n">
+      <c r="CJ5" t="n">
         <v>0.997707251307285</v>
       </c>
-      <c r="CH5" t="n">
-        <v>0.0430270852846958</v>
-      </c>
-      <c r="CI5" t="n">
-        <v>0.893669927958735</v>
+      <c r="CK5" t="n">
+        <v>0.00865559441587176</v>
+      </c>
+      <c r="CL5" t="n">
+        <v>4.44244616362096</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B6" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D6" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E6" t="n">
         <v>11.5</v>
@@ -2118,19 +2172,19 @@
         <v>9.4</v>
       </c>
       <c r="H6" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I6" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="J6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="K6" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="L6" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="M6" t="n">
         <v>600</v>
@@ -2139,10 +2193,10 @@
         <v>1.32386833098952</v>
       </c>
       <c r="O6" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="P6" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="Q6" t="n">
         <v>1.30314854895781</v>
@@ -2166,10 +2220,10 @@
         <v>0.704654629061883</v>
       </c>
       <c r="X6" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="Y6" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="Z6" t="n">
         <v>62</v>
@@ -2187,10 +2241,10 @@
         <v>0.353678991732009</v>
       </c>
       <c r="AE6" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="AF6" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="AG6" t="n">
         <v>0.330400946519775</v>
@@ -2214,10 +2268,10 @@
         <v>1.22995859003021</v>
       </c>
       <c r="AN6" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AO6" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AP6" t="n">
         <v>62</v>
@@ -2241,64 +2295,64 @@
         <v>62</v>
       </c>
       <c r="AW6" t="n">
+        <v>5</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>308</v>
+      </c>
+      <c r="AY6" t="n">
         <v>1.10388215394272</v>
       </c>
-      <c r="AX6" t="n">
+      <c r="AZ6" t="n">
         <v>1.24063893013517</v>
       </c>
-      <c r="AY6" t="n">
-        <v>62</v>
-      </c>
-      <c r="AZ6" t="n">
-        <v>0.0131755187787025</v>
-      </c>
       <c r="BA6" t="n">
-        <v>0.0338799054309493</v>
+        <v>1.04228663609991</v>
       </c>
       <c r="BB6" t="n">
-        <v>0.107038366282359</v>
+        <v>1.40029850566019</v>
       </c>
       <c r="BC6" t="n">
-        <v>0.120299040756893</v>
+        <v>0.00265221481908947</v>
       </c>
       <c r="BD6" t="n">
-        <v>0.0814461356536262</v>
+        <v>0.00681998096337291</v>
       </c>
       <c r="BE6" t="n">
-        <v>0.0915362624896662</v>
+        <v>0.0203444007425777</v>
       </c>
       <c r="BF6" t="n">
-        <v>0.0683517517096044</v>
+        <v>0.0273324371355108</v>
       </c>
       <c r="BG6" t="n">
-        <v>0.0768196530861471</v>
+        <v>0.0154801766901109</v>
       </c>
       <c r="BH6" t="n">
-        <v>0.146280124345726</v>
+        <v>0.020797415543607</v>
       </c>
       <c r="BI6" t="n">
-        <v>0.37329094553287</v>
+        <v>0.0129913738086131</v>
       </c>
       <c r="BJ6" t="n">
-        <v>0.109989730776377</v>
+        <v>0.0174537413227757</v>
       </c>
       <c r="BK6" t="n">
-        <v>0.280681813637105</v>
+        <v>0.0294459990566072</v>
       </c>
       <c r="BL6" t="n">
-        <v>0.0918634299604868</v>
+        <v>0.0751429825423309</v>
       </c>
       <c r="BM6" t="n">
-        <v>0.234425468143544</v>
-      </c>
-      <c r="BN6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP6" t="b">
-        <v>0</v>
+        <v>0.0221407899614785</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>0.0565008845633134</v>
+      </c>
+      <c r="BO6" t="n">
+        <v>0.0184919891478902</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>0.0471895422886355</v>
       </c>
       <c r="BQ6" t="b">
         <v>0</v>
@@ -2331,7 +2385,7 @@
         <v>0</v>
       </c>
       <c r="CA6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CB6" t="b">
         <v>0</v>
@@ -2340,36 +2394,45 @@
         <v>0</v>
       </c>
       <c r="CD6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CE6" t="b">
         <v>0</v>
       </c>
-      <c r="CF6" t="n">
+      <c r="CF6" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG6" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH6" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI6" t="n">
         <v>0.990407805013714</v>
       </c>
-      <c r="CG6" t="n">
+      <c r="CJ6" t="n">
         <v>0.999795764899988</v>
       </c>
-      <c r="CH6" t="n">
-        <v>0.0467733372081004</v>
-      </c>
-      <c r="CI6" t="n">
-        <v>7.56155136330015</v>
+      <c r="CK6" t="n">
+        <v>0.00941541203539683</v>
+      </c>
+      <c r="CL6" t="n">
+        <v>37.5638358047814</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B7" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C7" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="D7" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E7"/>
       <c r="F7"/>
@@ -2378,16 +2441,16 @@
       </c>
       <c r="H7"/>
       <c r="I7" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="J7" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="K7" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="L7" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="M7" t="n">
         <v>600</v>
@@ -2396,10 +2459,10 @@
         <v>1.34106207568664</v>
       </c>
       <c r="O7" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="P7" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="Q7" t="n">
         <v>1.31933987276378</v>
@@ -2423,10 +2486,10 @@
         <v>0.971891773133964</v>
       </c>
       <c r="X7" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="Y7" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="Z7" t="n">
         <v>117</v>
@@ -2444,10 +2507,10 @@
         <v>0.396629714787707</v>
       </c>
       <c r="AE7" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="AF7" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AG7" t="n">
         <v>0.369704402424142</v>
@@ -2471,10 +2534,10 @@
         <v>1.14932531698564</v>
       </c>
       <c r="AN7" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AO7" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AP7" t="n">
         <v>117</v>
@@ -2498,64 +2561,64 @@
         <v>117</v>
       </c>
       <c r="AW7" t="n">
+        <v>5</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>582</v>
+      </c>
+      <c r="AY7" t="n">
         <v>1.10388215394272</v>
       </c>
-      <c r="AX7" t="n">
+      <c r="AZ7" t="n">
         <v>1.24063893013517</v>
       </c>
-      <c r="AY7" t="n">
-        <v>117</v>
-      </c>
-      <c r="AZ7" t="n">
-        <v>0.00697950251157923</v>
-      </c>
       <c r="BA7" t="n">
-        <v>0.0179472921726323</v>
+        <v>1.04228663609991</v>
       </c>
       <c r="BB7" t="n">
-        <v>0.0567017176971174</v>
+        <v>1.40029850566019</v>
       </c>
       <c r="BC7" t="n">
-        <v>0.0637263299613308</v>
+        <v>0.00140309586572985</v>
       </c>
       <c r="BD7" t="n">
-        <v>0.0431446774810704</v>
+        <v>0.00360796079759103</v>
       </c>
       <c r="BE7" t="n">
-        <v>0.0484897471346564</v>
+        <v>0.0107627573630939</v>
       </c>
       <c r="BF7" t="n">
-        <v>0.0362081547406821</v>
+        <v>0.0144596241862196</v>
       </c>
       <c r="BG7" t="n">
-        <v>0.040693878598548</v>
+        <v>0.00818944670632634</v>
       </c>
       <c r="BH7" t="n">
-        <v>0.109775651159509</v>
+        <v>0.011002414871175</v>
       </c>
       <c r="BI7" t="n">
-        <v>0.17340174401312</v>
+        <v>0.0068728003289243</v>
       </c>
       <c r="BJ7" t="n">
-        <v>0.0830175718645747</v>
+        <v>0.00923351763033742</v>
       </c>
       <c r="BK7" t="n">
-        <v>0.131134651382159</v>
+        <v>0.022068301006293</v>
       </c>
       <c r="BL7" t="n">
-        <v>0.0694972716478955</v>
+        <v>0.0348591134871735</v>
       </c>
       <c r="BM7" t="n">
-        <v>0.109777969710132</v>
-      </c>
-      <c r="BN7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP7" t="b">
-        <v>0</v>
+        <v>0.0166890994985485</v>
+      </c>
+      <c r="BN7" t="n">
+        <v>0.0263621206386815</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>0.013971101001381</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>0.0220687671066761</v>
       </c>
       <c r="BQ7" t="b">
         <v>0</v>
@@ -2602,31 +2665,40 @@
       <c r="CE7" t="b">
         <v>0</v>
       </c>
-      <c r="CF7" t="n">
+      <c r="CF7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI7" t="n">
         <v>0.998122550225431</v>
       </c>
-      <c r="CG7" t="n">
+      <c r="CJ7" t="n">
         <v>0.999894443336438</v>
       </c>
-      <c r="CH7" t="n">
-        <v>0.0220675404115027</v>
-      </c>
-      <c r="CI7" t="n">
-        <v>17.9734445883676</v>
+      <c r="CK7" t="n">
+        <v>0.00443625812396188</v>
+      </c>
+      <c r="CL7" t="n">
+        <v>89.4063653882902</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C8" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D8" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E8" t="n">
         <v>11.4</v>
@@ -2639,16 +2711,16 @@
       </c>
       <c r="H8"/>
       <c r="I8" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="J8" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="K8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="L8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="M8" t="n">
         <v>600</v>
@@ -2657,10 +2729,10 @@
         <v>1.09834555739463</v>
       </c>
       <c r="O8" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="P8" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="Q8" t="n">
         <v>0.932800122520638</v>
@@ -2684,10 +2756,10 @@
         <v>1.1228647114697</v>
       </c>
       <c r="X8" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="Y8" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="Z8" t="n">
         <v>166</v>
@@ -2705,10 +2777,10 @@
         <v>0.0337112943119567</v>
       </c>
       <c r="AE8" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="AF8" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="AG8" t="n">
         <v>0.0336412225079778</v>
@@ -2732,10 +2804,10 @@
         <v>1.38367415839523</v>
       </c>
       <c r="AN8" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AO8" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AP8" t="n">
         <v>166</v>
@@ -2759,64 +2831,64 @@
         <v>166</v>
       </c>
       <c r="AW8" t="n">
+        <v>5</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>826</v>
+      </c>
+      <c r="AY8" t="n">
         <v>1.10388215394272</v>
       </c>
-      <c r="AX8" t="n">
+      <c r="AZ8" t="n">
         <v>1.24063893013517</v>
       </c>
-      <c r="AY8" t="n">
-        <v>166</v>
-      </c>
-      <c r="AZ8" t="n">
-        <v>0.00492132249443286</v>
-      </c>
       <c r="BA8" t="n">
-        <v>0.0126548292713988</v>
+        <v>1.04228663609991</v>
       </c>
       <c r="BB8" t="n">
-        <v>0.0399809926728813</v>
+        <v>1.40029850566019</v>
       </c>
       <c r="BC8" t="n">
-        <v>0.0449341225404025</v>
+        <v>0.000989030912924763</v>
       </c>
       <c r="BD8" t="n">
-        <v>0.0304217774046763</v>
+        <v>0.00254322234752082</v>
       </c>
       <c r="BE8" t="n">
-        <v>0.0341906436636772</v>
+        <v>0.00758658050415642</v>
       </c>
       <c r="BF8" t="n">
-        <v>0.0255307604104444</v>
+        <v>0.0101924719890802</v>
       </c>
       <c r="BG8" t="n">
-        <v>0.0286936926808899</v>
+        <v>0.00577267466189381</v>
       </c>
       <c r="BH8" t="n">
-        <v>0.0609877326793533</v>
+        <v>0.00775551314076094</v>
       </c>
       <c r="BI8" t="n">
-        <v>0.143252216155764</v>
+        <v>0.00484458129318898</v>
       </c>
       <c r="BJ8" t="n">
-        <v>0.0462071914551354</v>
+        <v>0.00650863180092774</v>
       </c>
       <c r="BK8" t="n">
-        <v>0.108534655864042</v>
+        <v>0.0122566145578361</v>
       </c>
       <c r="BL8" t="n">
-        <v>0.0387108138564723</v>
+        <v>0.0287891862976474</v>
       </c>
       <c r="BM8" t="n">
-        <v>0.0909266442694014</v>
-      </c>
-      <c r="BN8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP8" t="b">
-        <v>0</v>
+        <v>0.00928619101882867</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>0.0218120494835727</v>
+      </c>
+      <c r="BO8" t="n">
+        <v>0.0077796550849569</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>0.0182733934003882</v>
       </c>
       <c r="BQ8" t="b">
         <v>0</v>
@@ -2840,54 +2912,63 @@
         <v>0</v>
       </c>
       <c r="BX8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BY8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BZ8" t="b">
         <v>0</v>
       </c>
       <c r="CA8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CB8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CC8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CD8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CE8" t="b">
         <v>0</v>
       </c>
-      <c r="CF8" t="n">
+      <c r="CF8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI8" t="n">
         <v>0.859492457974167</v>
       </c>
-      <c r="CG8" t="n">
+      <c r="CJ8" t="n">
         <v>0.999860422432155</v>
       </c>
-      <c r="CH8" t="n">
-        <v>0.0183224031950001</v>
-      </c>
-      <c r="CI8" t="n">
-        <v>1.8398947972696</v>
+      <c r="CK8" t="n">
+        <v>0.00368222630795402</v>
+      </c>
+      <c r="CL8" t="n">
+        <v>9.15513917195598</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B9" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C9" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D9" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E9" t="n">
         <v>11.3</v>
@@ -2900,16 +2981,16 @@
       </c>
       <c r="H9"/>
       <c r="I9" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="J9" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="K9" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="L9" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="M9" t="n">
         <v>900</v>
@@ -2918,10 +2999,10 @@
         <v>1.25398474563604</v>
       </c>
       <c r="O9" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="P9" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="Q9" t="n">
         <v>1.10063846684457</v>
@@ -2945,10 +3026,10 @@
         <v>1.17849683682608</v>
       </c>
       <c r="X9" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="Y9" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="Z9" t="n">
         <v>192</v>
@@ -2966,10 +3047,10 @@
         <v>0.0765684447151247</v>
       </c>
       <c r="AE9" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="AF9" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="AG9" t="n">
         <v>0.0760943600684935</v>
@@ -2993,10 +3074,10 @@
         <v>1.56049523863239</v>
       </c>
       <c r="AN9" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AO9" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AP9" t="n">
         <v>192</v>
@@ -3020,64 +3101,64 @@
         <v>192</v>
       </c>
       <c r="AW9" t="n">
+        <v>5</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>954</v>
+      </c>
+      <c r="AY9" t="n">
         <v>1.10388215394272</v>
       </c>
-      <c r="AX9" t="n">
+      <c r="AZ9" t="n">
         <v>1.24063893013517</v>
       </c>
-      <c r="AY9" t="n">
-        <v>192</v>
-      </c>
-      <c r="AZ9" t="n">
-        <v>0.00425843595209661</v>
-      </c>
       <c r="BA9" t="n">
-        <v>0.0109502638768199</v>
+        <v>1.04228663609991</v>
       </c>
       <c r="BB9" t="n">
-        <v>0.0345956796758001</v>
+        <v>1.40029850566019</v>
       </c>
       <c r="BC9" t="n">
-        <v>0.0388816386486405</v>
+        <v>0.000857043713629507</v>
       </c>
       <c r="BD9" t="n">
-        <v>0.0263240604071982</v>
+        <v>0.00220382669219016</v>
       </c>
       <c r="BE9" t="n">
-        <v>0.0295852723261751</v>
+        <v>0.00657414348132317</v>
       </c>
       <c r="BF9" t="n">
-        <v>0.0220918479004759</v>
+        <v>0.00883227604964717</v>
       </c>
       <c r="BG9" t="n">
-        <v>0.0248287432187056</v>
+        <v>0.0050023052516871</v>
       </c>
       <c r="BH9" t="n">
-        <v>0.0568501845799588</v>
+        <v>0.00672053188267315</v>
       </c>
       <c r="BI9" t="n">
-        <v>0.109670233856289</v>
+        <v>0.0041980669039114</v>
       </c>
       <c r="BJ9" t="n">
-        <v>0.0430978645496238</v>
+        <v>0.00564004814856435</v>
       </c>
       <c r="BK9" t="n">
-        <v>0.0831405019840541</v>
+        <v>0.0114415465821301</v>
       </c>
       <c r="BL9" t="n">
-        <v>0.0361145757202873</v>
+        <v>0.0220719967509512</v>
       </c>
       <c r="BM9" t="n">
-        <v>0.0696689728296996</v>
-      </c>
-      <c r="BN9" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO9" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP9" t="b">
-        <v>0</v>
+        <v>0.00867378406030165</v>
+      </c>
+      <c r="BN9" t="n">
+        <v>0.0167326796445895</v>
+      </c>
+      <c r="BO9" t="n">
+        <v>0.00726834228332826</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>0.0140214284940276</v>
       </c>
       <c r="BQ9" t="b">
         <v>0</v>
@@ -3110,61 +3191,70 @@
         <v>0</v>
       </c>
       <c r="CA9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CB9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CC9" t="b">
         <v>0</v>
       </c>
       <c r="CD9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CE9" t="b">
         <v>0</v>
       </c>
-      <c r="CF9" t="n">
+      <c r="CF9" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG9" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH9" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI9" t="n">
         <v>0.97052787072339</v>
       </c>
-      <c r="CG9" t="n">
+      <c r="CJ9" t="n">
         <v>0.9999173464781</v>
       </c>
-      <c r="CH9" t="n">
-        <v>0.0140497362289817</v>
-      </c>
-      <c r="CI9" t="n">
-        <v>5.44981368099848</v>
+      <c r="CK9" t="n">
+        <v>0.00282761986998374</v>
+      </c>
+      <c r="CL9" t="n">
+        <v>27.0787617274612</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B10" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C10" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D10" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E10"/>
       <c r="F10"/>
       <c r="G10"/>
       <c r="H10"/>
       <c r="I10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="J10" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="K10" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="L10" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="M10" t="n">
         <v>300</v>
@@ -3173,10 +3263,10 @@
         <v>1.34102040741186</v>
       </c>
       <c r="O10" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="P10" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="Q10" t="n">
         <v>1.26070021803685</v>
@@ -3200,10 +3290,10 @@
         <v>1.13993468094949</v>
       </c>
       <c r="X10" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="Y10" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="Z10" t="n">
         <v>70</v>
@@ -3221,10 +3311,10 @@
         <v>0.00965562852738834</v>
       </c>
       <c r="AE10" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="AF10" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="AG10" t="n">
         <v>0.00966301603762399</v>
@@ -3248,10 +3338,10 @@
         <v>3.7919252851978</v>
       </c>
       <c r="AN10" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="AO10" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="AP10" t="n">
         <v>70</v>
@@ -3275,94 +3365,94 @@
         <v>70</v>
       </c>
       <c r="AW10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>575</v>
+      </c>
+      <c r="AY10" t="n">
         <v>1.10388215394272</v>
       </c>
-      <c r="AX10" t="n">
+      <c r="AZ10" t="n">
         <v>1.24063893013517</v>
       </c>
-      <c r="AY10" t="n">
-        <v>70</v>
-      </c>
-      <c r="AZ10" t="n">
-        <v>0.0116263382198069</v>
-      </c>
       <c r="BA10" t="n">
-        <v>0.0298962982795033</v>
+        <v>1.04228663609991</v>
       </c>
       <c r="BB10" t="n">
-        <v>0.0944527703080563</v>
+        <v>1.40029850566019</v>
       </c>
       <c r="BC10" t="n">
-        <v>0.106154251597196</v>
+        <v>0.00141538030501996</v>
       </c>
       <c r="BD10" t="n">
-        <v>0.0718696801021582</v>
+        <v>0.00363954935576562</v>
       </c>
       <c r="BE10" t="n">
-        <v>0.0807734074807096</v>
+        <v>0.0108569878733894</v>
       </c>
       <c r="BF10" t="n">
-        <v>0.0603149368643213</v>
+        <v>0.0145862216481693</v>
       </c>
       <c r="BG10" t="n">
-        <v>0.0677871804297734</v>
+        <v>0.0082611472674503</v>
       </c>
       <c r="BH10" t="n">
-        <v>2.6200523480139</v>
+        <v>0.0110987436401713</v>
       </c>
       <c r="BI10" t="n">
-        <v>0.638007459673722</v>
+        <v>0.00693297333666805</v>
       </c>
       <c r="BJ10" t="n">
-        <v>1.9728576107294</v>
+        <v>0.00931435928167043</v>
       </c>
       <c r="BK10" t="n">
-        <v>0.480409436656323</v>
+        <v>0.318962894540822</v>
       </c>
       <c r="BL10" t="n">
-        <v>1.648676465864</v>
+        <v>0.0776704733515835</v>
       </c>
       <c r="BM10" t="n">
-        <v>0.401468270130976</v>
-      </c>
-      <c r="BN10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP10" t="b">
-        <v>0</v>
+        <v>0.24017397000184</v>
+      </c>
+      <c r="BN10" t="n">
+        <v>0.0584846270712045</v>
+      </c>
+      <c r="BO10" t="n">
+        <v>0.200708439322574</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>0.0488743981029014</v>
       </c>
       <c r="BQ10" t="b">
         <v>0</v>
       </c>
       <c r="BR10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BS10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BT10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BU10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BV10" t="b">
         <v>0</v>
       </c>
       <c r="BW10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BX10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BY10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BZ10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CA10" t="b">
         <v>1</v>
@@ -3371,7 +3461,7 @@
         <v>1</v>
       </c>
       <c r="CC10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CD10" t="b">
         <v>1</v>
@@ -3379,17 +3469,26 @@
       <c r="CE10" t="b">
         <v>1</v>
       </c>
-      <c r="CF10" t="n">
+      <c r="CF10" t="b">
+        <v>1</v>
+      </c>
+      <c r="CG10" t="b">
+        <v>1</v>
+      </c>
+      <c r="CH10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI10" t="n">
         <v>0.0305018423219471</v>
       </c>
-      <c r="CG10" t="n">
+      <c r="CJ10" t="n">
         <v>0.999884540341955</v>
       </c>
-      <c r="CH10" t="n">
-        <v>0.0802500486793828</v>
-      </c>
-      <c r="CI10" t="n">
-        <v>0.120319285611461</v>
+      <c r="CK10" t="n">
+        <v>0.00976957114357704</v>
+      </c>
+      <c r="CL10" t="n">
+        <v>0.98833698895129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>